<commit_message>
Added soil parameters and method to classify soil texture
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Regions.xlsx
+++ b/data/prod_parameters/Regions.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>f_region</t>
   </si>
@@ -63,24 +63,15 @@
     <t>soil_sand</t>
   </si>
   <si>
-    <t>soil_carbon</t>
-  </si>
-  <si>
     <t>%</t>
   </si>
   <si>
     <t>clay content</t>
   </si>
   <si>
-    <t>silt content</t>
-  </si>
-  <si>
     <t>sand content</t>
   </si>
   <si>
-    <t>carbon content</t>
-  </si>
-  <si>
     <t>multiplied by land use in x0 to get maximum land use</t>
   </si>
   <si>
@@ -100,13 +91,40 @@
   </si>
   <si>
     <t>Regions_climate.csv</t>
+  </si>
+  <si>
+    <t>soil_OM</t>
+  </si>
+  <si>
+    <t>organic matter content (mullhalt)</t>
+  </si>
+  <si>
+    <t>silt content (finmo/mjäla)</t>
+  </si>
+  <si>
+    <t>Regions_soil.csv</t>
+  </si>
+  <si>
+    <t>soil_pH</t>
+  </si>
+  <si>
+    <t>soil pH</t>
+  </si>
+  <si>
+    <t>pH</t>
+  </si>
+  <si>
+    <t>Fallback (avg. for all regions w. data)</t>
+  </si>
+  <si>
+    <t>Can we find data for missing regions?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,6 +136,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -143,9 +175,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -470,10 +504,10 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -487,7 +521,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -501,71 +535,144 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
         <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>11</v>
       </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
       <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
         <v>15</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>12</v>
       </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>13</v>
       </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
         <v>14</v>
       </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
       <c r="F9" t="s">
-        <v>19</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2">
+        <v>20</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2">
+        <v>40</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="2">
+        <v>6.4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added parameter for share of organic soils
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Regions.xlsx
+++ b/data/prod_parameters/Regions.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t>f_region</t>
   </si>
@@ -118,13 +118,25 @@
   </si>
   <si>
     <t>Regions-soil.csv</t>
+  </si>
+  <si>
+    <t>share_org_soil</t>
+  </si>
+  <si>
+    <t>Regions-org_soil.csv</t>
+  </si>
+  <si>
+    <t>share organic soils based on county level data</t>
+  </si>
+  <si>
+    <t>Anna Lindahl och Mattias Lundblad (2021) Markanvändning på organogena jordar i Sverige</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,6 +166,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -175,11 +193,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -671,6 +690,23 @@
         <v>6.4</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C16" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Implemented paremeters to control land use constraints
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Regions.xlsx
+++ b/data/prod_parameters/Regions.xlsx
@@ -10,6 +10,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>f_region</t>
   </si>
@@ -42,9 +43,6 @@
     <t>f_land_use</t>
   </si>
   <si>
-    <t>land_use_factor</t>
-  </si>
-  <si>
     <t>cropland</t>
   </si>
   <si>
@@ -126,10 +124,19 @@
     <t>Regions-org_soil.csv</t>
   </si>
   <si>
-    <t>share organic soils based on county level data</t>
-  </si>
-  <si>
     <t>Anna Lindahl och Mattias Lundblad (2021) Markanvändning på organogena jordar i Sverige</t>
+  </si>
+  <si>
+    <t>max_land_use_factor</t>
+  </si>
+  <si>
+    <t>Climate and soil properties</t>
+  </si>
+  <si>
+    <t>Land use constraints</t>
+  </si>
+  <si>
+    <t>share organic soils calculated from county level data</t>
   </si>
 </sst>
 </file>
@@ -173,12 +180,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -193,12 +206,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -513,118 +528,112 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
       <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>20</v>
+        <v>35</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
         <v>13</v>
       </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>14</v>
-      </c>
-      <c r="F8" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
         <v>24</v>
@@ -632,93 +641,121 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" t="s">
         <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="2">
-        <v>20</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="2">
-        <v>40</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C13" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D13" s="2">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" s="2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D14" s="2">
-        <v>4.4000000000000004</v>
+        <v>40</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" s="2" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="2">
         <v>6.4</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C16" s="4" t="s">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" t="s">
         <v>33</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>38</v>
+      </c>
+      <c r="G18" t="s">
         <v>34</v>
       </c>
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="2">
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="2">
         <v>0</v>
       </c>
-      <c r="E17" t="s">
-        <v>14</v>
+      <c r="E19" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>